<commit_message>
Fixed colles index. Parafit not working
</commit_message>
<xml_diff>
--- a/parafit_summary_cosp.xlsx
+++ b/parafit_summary_cosp.xlsx
@@ -476,10 +476,10 @@
         <v>191</v>
       </c>
       <c r="E2" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>29.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -489,19 +489,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6346.29</v>
+        <v>16350.03</v>
       </c>
       <c r="C3" t="n">
-        <v>6565.9</v>
+        <v>15027.43</v>
       </c>
       <c r="D3" t="n">
-        <v>74</v>
+        <v>500</v>
       </c>
       <c r="E3" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -520,10 +520,10 @@
         <v>500</v>
       </c>
       <c r="E4" t="n">
-        <v>495</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -533,19 +533,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15807.72</v>
+        <v>205038484.64</v>
       </c>
       <c r="C5" t="n">
-        <v>21682.83</v>
+        <v>1164019159.73</v>
       </c>
       <c r="D5" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="E5" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>56.52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -564,10 +564,10 @@
         <v>497</v>
       </c>
       <c r="E6" t="n">
-        <v>425</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>85.51000000000001</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>